<commit_message>
edu, skoc42 @ 260424-134018
</commit_message>
<xml_diff>
--- a/csv/edu/events-contents.xlsx
+++ b/csv/edu/events-contents.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA560F51-A924-41D7-9C0A-C17172961541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F6699D4-5BFA-4C88-8913-F62F20C77982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="62">
   <si>
     <t>date</t>
   </si>
@@ -87,39 +88,99 @@
     <t>IM</t>
   </si>
   <si>
+    <t xml:space="preserve">Workshop 1 </t>
+  </si>
+  <si>
+    <t>Consumer analysis (group 1 + 2)</t>
+  </si>
+  <si>
+    <t>Chaffey &amp; Ellis-Chadwick ch. 2</t>
+  </si>
+  <si>
+    <t>Module 2: Plan</t>
+  </si>
+  <si>
+    <t>Lecture 4</t>
+  </si>
+  <si>
+    <t>Planning digital marketing</t>
+  </si>
+  <si>
+    <t>Chaffey &amp; Ellis-Chadwick ch. 7–8</t>
+  </si>
+  <si>
+    <t>Lecture 5</t>
+  </si>
+  <si>
+    <t>Implementing digital marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workshop 2 </t>
+  </si>
+  <si>
+    <t>Measuring digital marketing (group 1 + 2)</t>
+  </si>
+  <si>
+    <t>Team Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervision 1 </t>
+  </si>
+  <si>
+    <t>Project description review (group 1 + 2)</t>
+  </si>
+  <si>
+    <t>Module 3: Create</t>
+  </si>
+  <si>
+    <t>Lecture 6</t>
+  </si>
+  <si>
+    <t>Content marketing &amp; social media</t>
+  </si>
+  <si>
+    <t>Freberg Part II (ch. 7–13), Part III; storytelling article</t>
+  </si>
+  <si>
+    <t>Lecture 7</t>
+  </si>
+  <si>
+    <t>Brand storytelling &amp; Creative lab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervision 2 </t>
+  </si>
+  <si>
+    <t>Campaign review (group 1 + 2)</t>
+  </si>
+  <si>
+    <t>Examination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seminar </t>
+  </si>
+  <si>
+    <t>Team presentations (group 1 + 2)</t>
+  </si>
+  <si>
+    <t>Individual hall exam</t>
+  </si>
+  <si>
     <t>Workshop 1 (Grupp 1)</t>
   </si>
   <si>
     <t>Consumer analysis</t>
   </si>
   <si>
-    <t>Chaffey &amp; Ellis-Chadwick ch. 2</t>
-  </si>
-  <si>
     <t>Workshop 1 (Grupp 2)</t>
   </si>
   <si>
-    <t>Module 2: Plan</t>
-  </si>
-  <si>
-    <t>Lecture 4</t>
-  </si>
-  <si>
-    <t>Planning digital marketing</t>
-  </si>
-  <si>
-    <t>Chaffey &amp; Ellis-Chadwick ch. 7–8</t>
+    <t>SKDA50</t>
   </si>
   <si>
     <t>Information</t>
   </si>
   <si>
-    <t>Lecture 5</t>
-  </si>
-  <si>
-    <t>Implementing digital marketing</t>
-  </si>
-  <si>
     <t>Workshop 2 (Grupp 1)</t>
   </si>
   <si>
@@ -129,9 +190,6 @@
     <t>Workshop 2 (Grupp 2)</t>
   </si>
   <si>
-    <t>Team Project</t>
-  </si>
-  <si>
     <t>Supervision 1 (Grupp 1)</t>
   </si>
   <si>
@@ -141,24 +199,6 @@
     <t>Supervision 1 (Grupp 2)</t>
   </si>
   <si>
-    <t>Module 3: Create</t>
-  </si>
-  <si>
-    <t>Lecture 6</t>
-  </si>
-  <si>
-    <t>Content marketing &amp; social media</t>
-  </si>
-  <si>
-    <t>Freberg Part II (ch. 7–13), Part III; storytelling article</t>
-  </si>
-  <si>
-    <t>Lecture 7</t>
-  </si>
-  <si>
-    <t>Brand storytelling &amp; Creative lab</t>
-  </si>
-  <si>
     <t>Supervision 2 (Grupp 1)</t>
   </si>
   <si>
@@ -168,9 +208,6 @@
     <t>Supervision 2 (Grupp 2)</t>
   </si>
   <si>
-    <t>Examination</t>
-  </si>
-  <si>
     <t>Seminar (Grupp 1)</t>
   </si>
   <si>
@@ -181,9 +218,6 @@
   </si>
   <si>
     <t>Written examination</t>
-  </si>
-  <si>
-    <t>Individual hall exam</t>
   </si>
 </sst>
 </file>
@@ -544,6 +578,296 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2">
+        <v>46140</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2">
+        <v>46141</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="2">
+        <v>46148</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="2">
+        <v>46154</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2">
+        <v>46167</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2">
+        <v>46174</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2">
+        <v>46177</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95049E28-3784-4F83-845B-341F19FA0F95}">
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -635,16 +959,16 @@
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -655,16 +979,16 @@
         <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -672,16 +996,16 @@
         <v>46150</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>14</v>
@@ -692,10 +1016,10 @@
         <v>46150</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>9</v>
@@ -712,13 +1036,13 @@
         <v>46154</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>9</v>
@@ -732,13 +1056,13 @@
         <v>46155</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>9</v>
@@ -752,13 +1076,13 @@
         <v>46155</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>9</v>
@@ -772,19 +1096,19 @@
         <v>46161</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -792,19 +1116,19 @@
         <v>46161</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -812,16 +1136,16 @@
         <v>46162</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>17</v>
@@ -832,13 +1156,13 @@
         <v>46164</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>9</v>
@@ -852,19 +1176,19 @@
         <v>46167</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -872,19 +1196,19 @@
         <v>46167</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -892,19 +1216,19 @@
         <v>46174</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -912,19 +1236,19 @@
         <v>46174</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -932,19 +1256,19 @@
         <v>46177</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>